<commit_message>
Kinda working version of `run_montecarlo_simulation_class.py` & `montecarlo_simulation_class.py`
</commit_message>
<xml_diff>
--- a/Data/portfolio_by_Asset_class_2026_06_02.xlsx
+++ b/Data/portfolio_by_Asset_class_2026_06_02.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Asset_class</t>
   </si>
@@ -34,7 +34,22 @@
     <t>Non-US Emrg Stk</t>
   </si>
   <si>
-    <t>Real Estate</t>
+    <t>U.S. High Yield Bonds</t>
+  </si>
+  <si>
+    <t>U.S. Investment Grade Bonds</t>
+  </si>
+  <si>
+    <t>U.S. Lg Cap Val</t>
+  </si>
+  <si>
+    <t>U.S. Mid Cap Growth</t>
+  </si>
+  <si>
+    <t>U.S. Sm Cap Growth</t>
+  </si>
+  <si>
+    <t>U.S. Sm Cap Val</t>
   </si>
   <si>
     <t>US High Yield Bonds</t>
@@ -50,9 +65,6 @@
   </si>
   <si>
     <t>US Mid Cap Growth</t>
-  </si>
-  <si>
-    <t>US Mid Cap Value</t>
   </si>
   <si>
     <t>US Small Cap Growth</t>
@@ -425,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -473,7 +485,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>27515.6</v>
+        <v>120038.4</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -481,7 +493,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>14818.82</v>
+        <v>24460.52</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -489,7 +501,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>129068.78</v>
+        <v>75518.26999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -497,7 +509,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>618659.88</v>
+        <v>24923.75</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -505,7 +517,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>429838.52</v>
+        <v>102197.4</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -513,7 +525,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>263366.63</v>
+        <v>63452.4</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -521,7 +533,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>24619.87</v>
+        <v>14818.82</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -529,7 +541,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>189718.08</v>
+        <v>129068.78</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -537,7 +549,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>146460.38</v>
+        <v>618659.88</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -545,7 +557,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>291834.42</v>
+        <v>406455.72</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -553,7 +565,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>125504.97</v>
+        <v>238442.88</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -561,6 +573,38 @@
         <v>17</v>
       </c>
       <c r="B17">
+        <v>145654.08</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>24874.58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>147335.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>125504.97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21">
         <v>138845.48</v>
       </c>
     </row>

</xml_diff>